<commit_message>
Add ISO9806_conversion_template.xlsx, closes #1508
</commit_message>
<xml_diff>
--- a/IDEAS/Resources/Data/Fluid/PVTCollectors/ISO9806_conversion_template.xlsx
+++ b/IDEAS/Resources/Data/Fluid/PVTCollectors/ISO9806_conversion_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workdir\Develop\IDEAS\IDEAS\Resources\Data\Fluid\PVTCollectors\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E1371BB-B336-4553-85B3-A7CCCEB1D305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FDA755-99EA-4DBA-B16F-D13A2BB18F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-3510" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -378,9 +378,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="167" formatCode="0.0000"/>
-    <numFmt numFmtId="168" formatCode="0.000"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -682,17 +682,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -710,7 +707,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -720,26 +716,26 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -748,15 +744,12 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1256,84 +1249,75 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="120" style="51" customWidth="1"/>
-    <col min="2" max="6" width="8.88671875" style="51"/>
+    <col min="1" max="1" width="120" style="49" customWidth="1"/>
+    <col min="2" max="6" width="8.85546875" style="49"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="50" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="54" t="s">
+    <row r="2" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="54"/>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="53" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="54" t="s">
+    <row r="5" spans="1:1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="49" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="54" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="49" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="54" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="49" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="54" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="49" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="54"/>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="53" t="s">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="50" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="54" t="s">
+    <row r="11" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="49" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="54"/>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="55" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="51" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="56" t="s">
+    <row r="14" spans="1:1" ht="52.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="52" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52"/>
-    </row>
-    <row r="17" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" s="52"/>
-    </row>
-    <row r="20" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="50"/>
+    </row>
+    <row r="17" spans="1:1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="50"/>
+    </row>
+    <row r="20" spans="1:1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1342,17 +1326,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="C7:O30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="3:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C7" s="1"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -1367,222 +1351,222 @@
       <c r="N7" s="2"/>
       <c r="O7" s="3"/>
     </row>
-    <row r="8" spans="3:15" ht="31.2" x14ac:dyDescent="0.6">
+    <row r="8" spans="3:15" ht="31.5" x14ac:dyDescent="0.5">
       <c r="C8" s="4"/>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="6"/>
-    </row>
-    <row r="9" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E8" s="53"/>
+      <c r="F8" s="53"/>
+      <c r="G8" s="53"/>
+      <c r="H8" s="53"/>
+      <c r="I8" s="53"/>
+      <c r="J8" s="53"/>
+      <c r="K8" s="53"/>
+      <c r="L8" s="53"/>
+      <c r="M8" s="53"/>
+      <c r="N8" s="53"/>
+      <c r="O8" s="5"/>
+    </row>
+    <row r="9" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="4"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="6"/>
-    </row>
-    <row r="10" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="5"/>
+    </row>
+    <row r="10" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C10" s="4"/>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="7"/>
-      <c r="J10" s="11" t="s">
+      <c r="I10" s="6"/>
+      <c r="J10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="6"/>
-    </row>
-    <row r="11" spans="3:15" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="5"/>
+    </row>
+    <row r="11" spans="3:15" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="4"/>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="I11" s="7"/>
-      <c r="J11" s="15" t="s">
+      <c r="I11" s="6"/>
+      <c r="J11" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="6"/>
-    </row>
-    <row r="12" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="5"/>
+    </row>
+    <row r="12" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="4"/>
-      <c r="D12" s="16">
+      <c r="D12" s="15">
         <v>0.53500000000000003</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="16">
         <v>10.74</v>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="16">
         <v>1.0996999999999999</v>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="16">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="17">
         <v>0.85</v>
       </c>
-      <c r="I12" s="7"/>
-      <c r="J12" s="19">
+      <c r="I12" s="6"/>
+      <c r="J12" s="18">
         <v>22.1</v>
       </c>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="6"/>
-    </row>
-    <row r="13" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="5"/>
+    </row>
+    <row r="13" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="4"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="6"/>
-    </row>
-    <row r="14" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="5"/>
+    </row>
+    <row r="14" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C14" s="4"/>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="25">
         <v>10</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="25">
         <v>20</v>
       </c>
-      <c r="H14" s="27">
+      <c r="H14" s="25">
         <v>30</v>
       </c>
-      <c r="I14" s="27">
+      <c r="I14" s="25">
         <v>40</v>
       </c>
-      <c r="J14" s="27">
+      <c r="J14" s="25">
         <v>50</v>
       </c>
-      <c r="K14" s="27">
+      <c r="K14" s="25">
         <v>60</v>
       </c>
-      <c r="L14" s="27">
+      <c r="L14" s="25">
         <v>70</v>
       </c>
-      <c r="M14" s="27">
+      <c r="M14" s="25">
         <v>80</v>
       </c>
-      <c r="N14" s="28">
+      <c r="N14" s="26">
         <v>90</v>
       </c>
-      <c r="O14" s="6"/>
-    </row>
-    <row r="15" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O14" s="5"/>
+    </row>
+    <row r="15" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C15" s="4"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="26" t="s">
+      <c r="D15" s="11"/>
+      <c r="E15" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="17">
+      <c r="F15" s="16">
         <v>1</v>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="16">
         <v>1</v>
       </c>
-      <c r="H15" s="17">
+      <c r="H15" s="16">
         <v>1</v>
       </c>
-      <c r="I15" s="17">
+      <c r="I15" s="16">
         <v>0.99</v>
       </c>
-      <c r="J15" s="17">
+      <c r="J15" s="16">
         <v>0.97</v>
       </c>
-      <c r="K15" s="17">
+      <c r="K15" s="16">
         <v>0.92</v>
       </c>
-      <c r="L15" s="17">
+      <c r="L15" s="16">
         <v>0.8</v>
       </c>
-      <c r="M15" s="17">
+      <c r="M15" s="16">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N15" s="18">
+      <c r="N15" s="17">
         <v>0</v>
       </c>
-      <c r="O15" s="6"/>
-    </row>
-    <row r="16" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C16" s="20"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="22"/>
-    </row>
-    <row r="24" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="O15" s="5"/>
+    </row>
+    <row r="16" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C16" s="19"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="20"/>
+      <c r="M16" s="20"/>
+      <c r="N16" s="20"/>
+      <c r="O16" s="21"/>
+    </row>
+    <row r="24" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C24" s="1"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1597,165 +1581,165 @@
       <c r="N24" s="2"/>
       <c r="O24" s="3"/>
     </row>
-    <row r="25" spans="3:15" ht="31.2" x14ac:dyDescent="0.6">
+    <row r="25" spans="3:15" ht="31.5" x14ac:dyDescent="0.5">
       <c r="C25" s="4"/>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
-      <c r="N25" s="5"/>
-      <c r="O25" s="6"/>
-    </row>
-    <row r="26" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E25" s="53"/>
+      <c r="F25" s="53"/>
+      <c r="G25" s="53"/>
+      <c r="H25" s="53"/>
+      <c r="I25" s="53"/>
+      <c r="J25" s="53"/>
+      <c r="K25" s="53"/>
+      <c r="L25" s="53"/>
+      <c r="M25" s="53"/>
+      <c r="N25" s="53"/>
+      <c r="O25" s="5"/>
+    </row>
+    <row r="26" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C26" s="4"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7"/>
-      <c r="O26" s="6"/>
-    </row>
-    <row r="27" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="5"/>
+    </row>
+    <row r="27" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C27" s="4"/>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="H27" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="I27" s="9" t="s">
+      <c r="I27" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="J27" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="K27" s="9" t="s">
+      <c r="K27" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="L27" s="9" t="s">
+      <c r="L27" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="M27" s="10" t="s">
+      <c r="M27" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="N27" s="7"/>
-      <c r="O27" s="6"/>
-    </row>
-    <row r="28" spans="3:15" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N27" s="6"/>
+      <c r="O27" s="5"/>
+    </row>
+    <row r="28" spans="3:15" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="4"/>
-      <c r="D28" s="29" t="s">
+      <c r="D28" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="13" t="s">
+      <c r="F28" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="G28" s="13" t="s">
+      <c r="G28" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H28" s="25" t="s">
+      <c r="H28" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="I28" s="30" t="s">
+      <c r="I28" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="J28" s="13" t="s">
+      <c r="J28" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="K28" s="13" t="s">
+      <c r="K28" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="L28" s="13" t="s">
+      <c r="L28" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="M28" s="24" t="s">
+      <c r="M28" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="N28" s="7"/>
-      <c r="O28" s="6"/>
-    </row>
-    <row r="29" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N28" s="6"/>
+      <c r="O28" s="5"/>
+    </row>
+    <row r="29" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C29" s="4"/>
-      <c r="D29" s="31">
+      <c r="D29" s="29">
         <f>((1-3*G12)*D12)/(0.85+0.15*M29)</f>
         <v>0.43193348356348016</v>
       </c>
-      <c r="E29" s="32">
+      <c r="E29" s="30">
         <f>E12+3*F12</f>
         <v>14.039099999999999</v>
       </c>
-      <c r="F29" s="32">
+      <c r="F29" s="30">
         <v>0</v>
       </c>
-      <c r="G29" s="32">
+      <c r="G29" s="30">
         <f>F12</f>
         <v>1.0996999999999999</v>
       </c>
-      <c r="H29" s="33">
+      <c r="H29" s="31">
         <f>D12*H12*(1-3*G12)</f>
         <v>0.36334524999999995</v>
       </c>
-      <c r="I29" s="34">
+      <c r="I29" s="32">
         <f>J12*1000</f>
         <v>22100</v>
       </c>
-      <c r="J29" s="33">
+      <c r="J29" s="31">
         <f>D12*G12</f>
         <v>3.5845000000000002E-2</v>
       </c>
-      <c r="K29" s="35">
+      <c r="K29" s="33">
         <f>D12*G12*H12</f>
         <v>3.0468250000000002E-2</v>
       </c>
-      <c r="L29" s="36">
+      <c r="L29" s="34">
         <v>0</v>
       </c>
-      <c r="M29" s="37" cm="1">
+      <c r="M29" s="35" cm="1">
         <f t="array" ref="M29">SUMPRODUCT(F15:N15, SIN(RADIANS(F14:N14)), COS(RADIANS(F14:N14))) / SUMPRODUCT(SIN(RADIANS(F14:N14)), COS(RADIANS(F14:N14)))</f>
         <v>0.93103130098312248</v>
       </c>
-      <c r="N29" s="7"/>
-      <c r="O29" s="6"/>
-    </row>
-    <row r="30" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C30" s="20"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="21"/>
-      <c r="M30" s="21"/>
-      <c r="N30" s="21"/>
-      <c r="O30" s="22"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="5"/>
+    </row>
+    <row r="30" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C30" s="19"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
+      <c r="L30" s="20"/>
+      <c r="M30" s="20"/>
+      <c r="N30" s="20"/>
+      <c r="O30" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1770,9 +1754,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="C6:O29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="6" spans="3:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1787,234 +1771,234 @@
       <c r="N6" s="2"/>
       <c r="O6" s="3"/>
     </row>
-    <row r="7" spans="3:15" ht="31.2" x14ac:dyDescent="0.6">
+    <row r="7" spans="3:15" ht="31.5" x14ac:dyDescent="0.5">
       <c r="C7" s="4"/>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="6"/>
-    </row>
-    <row r="8" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="53"/>
+      <c r="I7" s="53"/>
+      <c r="J7" s="53"/>
+      <c r="K7" s="53"/>
+      <c r="L7" s="53"/>
+      <c r="M7" s="53"/>
+      <c r="N7" s="53"/>
+      <c r="O7" s="5"/>
+    </row>
+    <row r="8" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="4"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="6"/>
-    </row>
-    <row r="9" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="5"/>
+    </row>
+    <row r="9" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C9" s="4"/>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="7"/>
-      <c r="L9" s="11" t="s">
+      <c r="K9" s="6"/>
+      <c r="L9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="6"/>
-    </row>
-    <row r="10" spans="3:15" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="5"/>
+    </row>
+    <row r="10" spans="3:15" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="4"/>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="J10" s="24" t="s">
+      <c r="J10" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="15" t="s">
+      <c r="K10" s="6"/>
+      <c r="L10" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="M10" s="7"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="6"/>
-    </row>
-    <row r="11" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="5"/>
+    </row>
+    <row r="11" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="4"/>
-      <c r="D11" s="16">
+      <c r="D11" s="15">
         <v>0.47499999999999998</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="16">
         <v>7.4109999999999996</v>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="16">
         <v>0</v>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="16">
         <v>1.7</v>
       </c>
-      <c r="H11" s="17">
+      <c r="H11" s="16">
         <v>0.437</v>
       </c>
-      <c r="I11" s="17">
+      <c r="I11" s="16">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="17">
         <v>1</v>
       </c>
-      <c r="K11" s="7"/>
-      <c r="L11" s="19">
+      <c r="K11" s="6"/>
+      <c r="L11" s="18">
         <v>42.2</v>
       </c>
-      <c r="M11" s="7"/>
-      <c r="N11" s="23"/>
-      <c r="O11" s="6"/>
-    </row>
-    <row r="12" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="5"/>
+    </row>
+    <row r="12" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="4"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="6"/>
-    </row>
-    <row r="13" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="5"/>
+    </row>
+    <row r="13" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C13" s="4"/>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="8">
         <v>10</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="8">
         <v>20</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <v>30</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="8">
         <v>40</v>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="8">
         <v>50</v>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="8">
         <v>60</v>
       </c>
-      <c r="L13" s="9">
+      <c r="L13" s="8">
         <v>70</v>
       </c>
-      <c r="M13" s="9">
+      <c r="M13" s="8">
         <v>80</v>
       </c>
-      <c r="N13" s="10">
+      <c r="N13" s="9">
         <v>90</v>
       </c>
-      <c r="O13" s="6"/>
-    </row>
-    <row r="14" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O13" s="5"/>
+    </row>
+    <row r="14" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C14" s="4"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="14" t="s">
+      <c r="D14" s="11"/>
+      <c r="E14" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="38">
+      <c r="F14" s="36">
         <v>1</v>
       </c>
-      <c r="G14" s="38">
+      <c r="G14" s="36">
         <v>1</v>
       </c>
-      <c r="H14" s="38">
+      <c r="H14" s="36">
         <v>0.99</v>
       </c>
-      <c r="I14" s="38">
+      <c r="I14" s="36">
         <v>0.99</v>
       </c>
-      <c r="J14" s="38">
+      <c r="J14" s="36">
         <v>0.98</v>
       </c>
-      <c r="K14" s="38">
+      <c r="K14" s="36">
         <v>0.96</v>
       </c>
-      <c r="L14" s="38">
+      <c r="L14" s="36">
         <v>0.92</v>
       </c>
-      <c r="M14" s="38">
+      <c r="M14" s="36">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N14" s="39">
+      <c r="N14" s="37">
         <v>0</v>
       </c>
-      <c r="O14" s="6"/>
-    </row>
-    <row r="15" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C15" s="20"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21"/>
-      <c r="L15" s="21"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="21"/>
-      <c r="O15" s="22"/>
-    </row>
-    <row r="23" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="O14" s="5"/>
+    </row>
+    <row r="15" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C15" s="19"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
+      <c r="M15" s="20"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="21"/>
+    </row>
+    <row r="23" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C23" s="1"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -2029,165 +2013,165 @@
       <c r="N23" s="2"/>
       <c r="O23" s="3"/>
     </row>
-    <row r="24" spans="3:15" ht="31.2" x14ac:dyDescent="0.6">
+    <row r="24" spans="3:15" ht="31.5" x14ac:dyDescent="0.5">
       <c r="C24" s="4"/>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="5"/>
-      <c r="O24" s="6"/>
-    </row>
-    <row r="25" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
+      <c r="J24" s="53"/>
+      <c r="K24" s="53"/>
+      <c r="L24" s="53"/>
+      <c r="M24" s="53"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="5"/>
+    </row>
+    <row r="25" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C25" s="4"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
-      <c r="M25" s="7"/>
-      <c r="N25" s="7"/>
-      <c r="O25" s="6"/>
-    </row>
-    <row r="26" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="5"/>
+    </row>
+    <row r="26" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C26" s="4"/>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="40" t="s">
+      <c r="E26" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="F26" s="40" t="s">
+      <c r="F26" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="G26" s="40" t="s">
+      <c r="G26" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="H26" s="40" t="s">
+      <c r="H26" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="I26" s="40" t="s">
+      <c r="I26" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="J26" s="40" t="s">
+      <c r="J26" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="K26" s="40" t="s">
+      <c r="K26" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="L26" s="40" t="s">
+      <c r="L26" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="M26" s="41" t="s">
+      <c r="M26" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="N26" s="7"/>
-      <c r="O26" s="6"/>
-    </row>
-    <row r="27" spans="3:15" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N26" s="6"/>
+      <c r="O26" s="5"/>
+    </row>
+    <row r="27" spans="3:15" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C27" s="4"/>
-      <c r="D27" s="29" t="s">
+      <c r="D27" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="E27" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="13" t="s">
+      <c r="F27" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="G27" s="13" t="s">
+      <c r="G27" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H27" s="25" t="s">
+      <c r="H27" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="I27" s="30" t="s">
+      <c r="I27" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="J27" s="13" t="s">
+      <c r="J27" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="K27" s="13" t="s">
+      <c r="K27" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="L27" s="13" t="s">
+      <c r="L27" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="M27" s="24" t="s">
+      <c r="M27" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="N27" s="7"/>
-      <c r="O27" s="6"/>
-    </row>
-    <row r="28" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N27" s="6"/>
+      <c r="O27" s="5"/>
+    </row>
+    <row r="28" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="4"/>
-      <c r="D28" s="42">
+      <c r="D28" s="40">
         <f>D11-3*I11</f>
         <v>0.46599999999999997</v>
       </c>
-      <c r="E28" s="43">
+      <c r="E28" s="41">
         <f>E11+3*G11</f>
         <v>12.510999999999999</v>
       </c>
-      <c r="F28" s="43">
+      <c r="F28" s="41">
         <f>F11</f>
         <v>0</v>
       </c>
-      <c r="G28" s="43">
+      <c r="G28" s="41">
         <f>G11</f>
         <v>1.7</v>
       </c>
-      <c r="H28" s="44">
+      <c r="H28" s="42">
         <f>H11</f>
         <v>0.437</v>
       </c>
-      <c r="I28" s="45">
+      <c r="I28" s="43">
         <f>L11*1000</f>
         <v>42200</v>
       </c>
-      <c r="J28" s="44">
+      <c r="J28" s="42">
         <f>I11</f>
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="K28" s="47">
+      <c r="K28" s="45">
         <v>0</v>
       </c>
-      <c r="L28" s="47">
+      <c r="L28" s="45">
         <v>0</v>
       </c>
-      <c r="M28" s="46">
+      <c r="M28" s="44">
         <f>J11</f>
         <v>1</v>
       </c>
-      <c r="N28" s="7"/>
-      <c r="O28" s="6"/>
-    </row>
-    <row r="29" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C29" s="20"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="21"/>
-      <c r="I29" s="21"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="21"/>
-      <c r="L29" s="21"/>
-      <c r="M29" s="21"/>
-      <c r="N29" s="21"/>
-      <c r="O29" s="22"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="5"/>
+    </row>
+    <row r="29" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C29" s="19"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="20"/>
+      <c r="M29" s="20"/>
+      <c r="N29" s="20"/>
+      <c r="O29" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2202,9 +2186,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C46E3562-EEAB-4DA2-96EE-8007816CB685}">
   <dimension ref="C6:O29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="6" spans="3:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -2219,240 +2203,240 @@
       <c r="N6" s="2"/>
       <c r="O6" s="3"/>
     </row>
-    <row r="7" spans="3:15" ht="31.2" x14ac:dyDescent="0.6">
+    <row r="7" spans="3:15" ht="31.5" x14ac:dyDescent="0.5">
       <c r="C7" s="4"/>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="6"/>
-    </row>
-    <row r="8" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="53"/>
+      <c r="I7" s="53"/>
+      <c r="J7" s="53"/>
+      <c r="K7" s="53"/>
+      <c r="L7" s="53"/>
+      <c r="M7" s="53"/>
+      <c r="N7" s="53"/>
+      <c r="O7" s="5"/>
+    </row>
+    <row r="8" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="4"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="6"/>
-    </row>
-    <row r="9" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="5"/>
+    </row>
+    <row r="9" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C9" s="4"/>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="J9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="K9" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="L9" s="10" t="s">
+      <c r="L9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="48"/>
-      <c r="O9" s="6"/>
-    </row>
-    <row r="10" spans="3:15" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M9" s="6"/>
+      <c r="N9" s="46"/>
+      <c r="O9" s="5"/>
+    </row>
+    <row r="10" spans="3:15" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="4"/>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="I10" s="30" t="s">
+      <c r="I10" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="J10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="K10" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="L10" s="14" t="s">
+      <c r="L10" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="M10" s="7"/>
-      <c r="N10" s="50"/>
-      <c r="O10" s="6"/>
-    </row>
-    <row r="11" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M10" s="6"/>
+      <c r="N10" s="48"/>
+      <c r="O10" s="5"/>
+    </row>
+    <row r="11" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="4"/>
-      <c r="D11" s="16">
+      <c r="D11" s="15">
         <v>0.32900000000000001</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="16">
         <v>40.94</v>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="16">
         <v>0</v>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="16">
         <v>4.9279999999999999</v>
       </c>
-      <c r="H11" s="17">
+      <c r="H11" s="16">
         <v>0.14000000000000001</v>
       </c>
-      <c r="I11" s="17">
+      <c r="I11" s="16">
         <v>42730</v>
       </c>
-      <c r="J11" s="17">
+      <c r="J11" s="16">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="K11" s="17">
+      <c r="K11" s="16">
         <v>0</v>
       </c>
-      <c r="L11" s="18">
+      <c r="L11" s="17">
         <v>0.83</v>
       </c>
-      <c r="M11" s="7"/>
-      <c r="N11" s="49"/>
-      <c r="O11" s="6"/>
-    </row>
-    <row r="12" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M11" s="6"/>
+      <c r="N11" s="47"/>
+      <c r="O11" s="5"/>
+    </row>
+    <row r="12" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="4"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="6"/>
-    </row>
-    <row r="13" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="5"/>
+    </row>
+    <row r="13" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C13" s="4"/>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="8">
         <v>10</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="8">
         <v>20</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <v>30</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="8">
         <v>40</v>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="8">
         <v>50</v>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="8">
         <v>60</v>
       </c>
-      <c r="L13" s="9">
+      <c r="L13" s="8">
         <v>70</v>
       </c>
-      <c r="M13" s="9">
+      <c r="M13" s="8">
         <v>80</v>
       </c>
-      <c r="N13" s="10">
+      <c r="N13" s="9">
         <v>90</v>
       </c>
-      <c r="O13" s="6"/>
-    </row>
-    <row r="14" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O13" s="5"/>
+    </row>
+    <row r="14" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C14" s="4"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="14" t="s">
+      <c r="D14" s="11"/>
+      <c r="E14" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="38">
+      <c r="F14" s="36">
         <v>1</v>
       </c>
-      <c r="G14" s="38">
+      <c r="G14" s="36">
         <v>1</v>
       </c>
-      <c r="H14" s="17">
+      <c r="H14" s="16">
         <v>0.99</v>
       </c>
-      <c r="I14" s="38">
+      <c r="I14" s="36">
         <v>0.99</v>
       </c>
-      <c r="J14" s="38">
+      <c r="J14" s="36">
         <v>0.98</v>
       </c>
-      <c r="K14" s="38">
+      <c r="K14" s="36">
         <v>0.96</v>
       </c>
-      <c r="L14" s="38">
+      <c r="L14" s="36">
         <v>0.92</v>
       </c>
-      <c r="M14" s="38">
+      <c r="M14" s="36">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N14" s="39">
+      <c r="N14" s="37">
         <v>0</v>
       </c>
-      <c r="O14" s="6"/>
-    </row>
-    <row r="15" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C15" s="20"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21"/>
-      <c r="L15" s="21"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="21"/>
-      <c r="O15" s="22"/>
-    </row>
-    <row r="23" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="O14" s="5"/>
+    </row>
+    <row r="15" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C15" s="19"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
+      <c r="M15" s="20"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="21"/>
+    </row>
+    <row r="23" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C23" s="1"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -2467,166 +2451,166 @@
       <c r="N23" s="2"/>
       <c r="O23" s="3"/>
     </row>
-    <row r="24" spans="3:15" ht="31.2" x14ac:dyDescent="0.6">
+    <row r="24" spans="3:15" ht="31.5" x14ac:dyDescent="0.5">
       <c r="C24" s="4"/>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="5"/>
-      <c r="O24" s="6"/>
-    </row>
-    <row r="25" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
+      <c r="J24" s="53"/>
+      <c r="K24" s="53"/>
+      <c r="L24" s="53"/>
+      <c r="M24" s="53"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="5"/>
+    </row>
+    <row r="25" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C25" s="4"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
-      <c r="M25" s="7"/>
-      <c r="N25" s="7"/>
-      <c r="O25" s="6"/>
-    </row>
-    <row r="26" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="5"/>
+    </row>
+    <row r="26" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C26" s="4"/>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="I26" s="9" t="s">
+      <c r="I26" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="J26" s="9" t="s">
+      <c r="J26" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="K26" s="9" t="s">
+      <c r="K26" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="L26" s="9" t="s">
+      <c r="L26" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="M26" s="10" t="s">
+      <c r="M26" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="N26" s="7"/>
-      <c r="O26" s="6"/>
-    </row>
-    <row r="27" spans="3:15" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N26" s="6"/>
+      <c r="O26" s="5"/>
+    </row>
+    <row r="27" spans="3:15" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C27" s="4"/>
-      <c r="D27" s="29" t="s">
+      <c r="D27" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="E27" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="13" t="s">
+      <c r="F27" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="G27" s="13" t="s">
+      <c r="G27" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H27" s="25" t="s">
+      <c r="H27" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="I27" s="30" t="s">
+      <c r="I27" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="J27" s="13" t="s">
+      <c r="J27" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="K27" s="13" t="s">
+      <c r="K27" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="L27" s="13" t="s">
+      <c r="L27" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="M27" s="24" t="s">
+      <c r="M27" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="N27" s="7"/>
-      <c r="O27" s="6"/>
-    </row>
-    <row r="28" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N27" s="6"/>
+      <c r="O27" s="5"/>
+    </row>
+    <row r="28" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="4"/>
-      <c r="D28" s="42">
-        <f>D11</f>
-        <v>0.32900000000000001</v>
-      </c>
-      <c r="E28" s="43">
-        <f>E11</f>
-        <v>40.94</v>
-      </c>
-      <c r="F28" s="43">
-        <f>F11</f>
+      <c r="D28" s="40">
+        <f>D11-3*J11</f>
+        <v>0.19400000000000001</v>
+      </c>
+      <c r="E28" s="41">
+        <f>E11+3*G11</f>
+        <v>55.723999999999997</v>
+      </c>
+      <c r="F28" s="41">
+        <f t="shared" ref="D28:I28" si="0">F11</f>
         <v>0</v>
       </c>
-      <c r="G28" s="43">
-        <f>G11</f>
+      <c r="G28" s="41">
+        <f t="shared" si="0"/>
         <v>4.9279999999999999</v>
       </c>
-      <c r="H28" s="44">
-        <f>H11</f>
+      <c r="H28" s="42">
+        <f t="shared" si="0"/>
         <v>0.14000000000000001</v>
       </c>
-      <c r="I28" s="45">
-        <f>I11</f>
+      <c r="I28" s="43">
+        <f t="shared" si="0"/>
         <v>42730</v>
       </c>
-      <c r="J28" s="44">
+      <c r="J28" s="42">
         <f>(H14*850 + L11*150)/1000 * J11</f>
         <v>4.3469999999999995E-2</v>
       </c>
-      <c r="K28" s="47">
+      <c r="K28" s="45">
         <v>0</v>
       </c>
-      <c r="L28" s="47">
+      <c r="L28" s="45">
         <f>K11</f>
         <v>0</v>
       </c>
-      <c r="M28" s="46">
+      <c r="M28" s="44">
         <f>J11</f>
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="N28" s="7"/>
-      <c r="O28" s="6"/>
-    </row>
-    <row r="29" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C29" s="20"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="21"/>
-      <c r="I29" s="21"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="21"/>
-      <c r="L29" s="21"/>
-      <c r="M29" s="21"/>
-      <c r="N29" s="21"/>
-      <c r="O29" s="22"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="5"/>
+    </row>
+    <row r="29" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C29" s="19"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="20"/>
+      <c r="M29" s="20"/>
+      <c r="N29" s="20"/>
+      <c r="O29" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>